<commit_message>
update bug status and example codes
</commit_message>
<xml_diff>
--- a/uncovered_bugs/unconvered_bugs.xlsx
+++ b/uncovered_bugs/unconvered_bugs.xlsx
@@ -22,15 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="205">
   <si>
     <t>Status</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>still unconfirmed</t>
-  </si>
-  <si>
     <t>confirmed</t>
   </si>
   <si>
@@ -608,16 +605,55 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>fixed</t>
+    <t>no response yet</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>fixed</t>
+    <t>under discussion</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>fixed</t>
+    <t>invalid</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>not planned</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>invalid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>under discussion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>confirmed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>confirmed(already fixed)</t>
   </si>
 </sst>
 </file>
@@ -1103,1142 +1139,1142 @@
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" style="1" customWidth="1"/>
     <col min="3" max="3" width="30.6328125" style="1" customWidth="1"/>
     <col min="4" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>1</v>
+        <v>194</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>1</v>
+        <v>195</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>1</v>
+        <v>194</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>1</v>
+        <v>197</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>1</v>
+        <v>197</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>1</v>
+        <v>198</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>1</v>
+        <v>199</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>1</v>
+        <v>201</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>1</v>
+        <v>194</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>1</v>
+        <v>202</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
disable anonymization of bug report ids
</commit_message>
<xml_diff>
--- a/uncovered_bugs/unconvered_bugs.xlsx
+++ b/uncovered_bugs/unconvered_bugs.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="219">
   <si>
     <t>Status</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -35,270 +35,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>GCC-11XX76</t>
-  </si>
-  <si>
-    <t>GCC-11XX65</t>
-  </si>
-  <si>
-    <t>GCC-11XX08</t>
-  </si>
-  <si>
-    <t>GCC-11XX15</t>
-  </si>
-  <si>
-    <t>GCC-11XX16</t>
-  </si>
-  <si>
-    <t>GCC-11XX27</t>
-  </si>
-  <si>
-    <t>GCC-11XX11</t>
-  </si>
-  <si>
-    <t>GCC-11XX38</t>
-  </si>
-  <si>
-    <t>GCC-11XX85</t>
-  </si>
-  <si>
-    <t>GCC-11XX12</t>
-  </si>
-  <si>
-    <t>GCC-11XX44</t>
-  </si>
-  <si>
-    <t>LLVM-9XX53</t>
-  </si>
-  <si>
-    <t>GCC-11XX53</t>
-  </si>
-  <si>
-    <t>LLVM-9XX21</t>
-  </si>
-  <si>
-    <t>LLVM-9XX66</t>
-  </si>
-  <si>
-    <t>GCC-11XX83</t>
-  </si>
-  <si>
-    <t>LLVM-9XX32</t>
-  </si>
-  <si>
-    <t>LLVM-9XX04</t>
-  </si>
-  <si>
-    <t>LLVM-9XX89</t>
-  </si>
-  <si>
-    <t>LLVM-9XX91</t>
-  </si>
-  <si>
-    <t>LLVM-9XX49</t>
-  </si>
-  <si>
-    <t>GCC-11XX52</t>
-  </si>
-  <si>
-    <t>LLVM-9XX45</t>
-  </si>
-  <si>
-    <t>LLVM-10XX89</t>
-  </si>
-  <si>
-    <t>LLVM-10XX30</t>
-  </si>
-  <si>
-    <t>LLVM-10XX47</t>
-  </si>
-  <si>
-    <t>LLVM-10XX74</t>
-  </si>
-  <si>
-    <t>LLVM-10XX06</t>
-  </si>
-  <si>
-    <t>LLVM-10XX29</t>
-  </si>
-  <si>
-    <t>LLVM-10XX81</t>
-  </si>
-  <si>
-    <t>LLVM-10XX14</t>
-  </si>
-  <si>
-    <t>LLVM-10XX67</t>
-  </si>
-  <si>
-    <t>GCC-11XX32</t>
-  </si>
-  <si>
-    <t>GCC-11XX80</t>
-  </si>
-  <si>
-    <t>LLVM-12XX39</t>
-  </si>
-  <si>
-    <t>GCC-11XX90</t>
-  </si>
-  <si>
-    <t>GCC-11XX92</t>
-  </si>
-  <si>
-    <t>GCC-11XX93</t>
-  </si>
-  <si>
-    <t>GCC-11XX01</t>
-  </si>
-  <si>
-    <t>GCC-11XX02</t>
-  </si>
-  <si>
-    <t>LLVM-12XX55</t>
-  </si>
-  <si>
-    <t>GCC-11XX18</t>
-  </si>
-  <si>
-    <t>GCC-11XX25</t>
-  </si>
-  <si>
-    <t>LLVM-12XX58</t>
-  </si>
-  <si>
-    <t>GCC-11XX28</t>
-  </si>
-  <si>
-    <t>GCC-11XX36</t>
-  </si>
-  <si>
-    <t>GCC-11XX40</t>
-  </si>
-  <si>
-    <t>LLVM-12XX19</t>
-  </si>
-  <si>
-    <t>GCC-11XX42</t>
-  </si>
-  <si>
-    <t>LLVM-12XX31</t>
-  </si>
-  <si>
-    <t>LLVM-12XX34</t>
-  </si>
-  <si>
-    <t>GCC-11XX55</t>
-  </si>
-  <si>
-    <t>LLVM-12XX81</t>
-  </si>
-  <si>
-    <t>GCC-11XX56</t>
-  </si>
-  <si>
-    <t>GCC-11XX62</t>
-  </si>
-  <si>
-    <t>GCC-11XX64</t>
-  </si>
-  <si>
-    <t>LLVM-12XX29</t>
-  </si>
-  <si>
-    <t>GCC-11XX71</t>
-  </si>
-  <si>
-    <t>LLVM-12XX53</t>
-  </si>
-  <si>
-    <t>GCC-11XX82</t>
-  </si>
-  <si>
-    <t>LLVM-12XX45</t>
-  </si>
-  <si>
-    <t>GCC-11XX19</t>
-  </si>
-  <si>
-    <t>LLVM-12XX82</t>
-  </si>
-  <si>
-    <t>GCC-11XX24</t>
-  </si>
-  <si>
-    <t>LLVM-12XX24</t>
-  </si>
-  <si>
-    <t>GCC-11XX47</t>
-  </si>
-  <si>
-    <t>GCC-11XX46</t>
-  </si>
-  <si>
-    <t>GCC-11XX81</t>
-  </si>
-  <si>
-    <t>GCC-11XX94</t>
-  </si>
-  <si>
-    <t>LLVM-12XX79</t>
-  </si>
-  <si>
-    <t>GCC-11XX35</t>
-  </si>
-  <si>
-    <t>GCC-11XX07</t>
-  </si>
-  <si>
-    <t>LLVM-12XX00</t>
-  </si>
-  <si>
-    <t>GCC-11XX77</t>
-  </si>
-  <si>
-    <t>LLVM-13XX49</t>
-  </si>
-  <si>
-    <t>LLVM-13XX51</t>
-  </si>
-  <si>
-    <t>LLVM-13XX56</t>
-  </si>
-  <si>
-    <t>LLVM-13XX57</t>
-  </si>
-  <si>
-    <t>LLVM-13XX44</t>
-  </si>
-  <si>
-    <t>LLVM-13XX13</t>
-  </si>
-  <si>
-    <t>LLVM-13XX14</t>
-  </si>
-  <si>
-    <t>LLVM-13XX16</t>
-  </si>
-  <si>
-    <t>GCC-11XX37</t>
-  </si>
-  <si>
-    <t>GCC-11XX48</t>
-  </si>
-  <si>
-    <t>GCC-11XX45</t>
-  </si>
-  <si>
-    <t>LLVM-13XX71</t>
-  </si>
-  <si>
-    <t>LLVM-13XX73</t>
-  </si>
-  <si>
-    <t>GCC-11XX51</t>
-  </si>
-  <si>
     <t>https://godbolt.org/z/Po5xTqvPn</t>
   </si>
   <si>
@@ -654,6 +390,414 @@
   </si>
   <si>
     <t>confirmed(already fixed)</t>
+  </si>
+  <si>
+    <t>GCC-115676</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115665</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115708</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115715</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115716</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115727</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115911</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115915</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115938</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-115985</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-116012</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-116144</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-96753</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119453</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-97021</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-97266</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118383</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-97532</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-98804</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-98889</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-99491</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-99749</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119452</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-99845</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101189</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101330</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101347</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118385</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101674</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101806</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101829</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-101881</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-102314</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-102467</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-102589</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119032</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118180</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-120939</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118190</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118192</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118193</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118201</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118202</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121155</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118218</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118225</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121258</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118228</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118236</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118240</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121319</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118242</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121331</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121334</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118255</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121381</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118256</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118262</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118264</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121429</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118271</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121553</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118282</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118292</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121645</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118302</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118312</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118319</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121882</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118324</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-121924</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118347</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118346</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118382</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118381</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118394</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118393</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-122579</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118428</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118435</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118507</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118576</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-123700</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-118577</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119392</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132249</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132251</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132256</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132257</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132344</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132613</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132614</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132616</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119436</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119437</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119448</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119445</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119446</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119447</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132771</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LLVM-132773</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GCC-119451</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1152,1129 +1296,1129 @@
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>130</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>5</v>
+        <v>119</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>98</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>6</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>9</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>6</v>
+        <v>124</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>93</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>99</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>194</v>
+        <v>106</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>13</v>
+        <v>128</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>102</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>14</v>
+        <v>129</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>103</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>15</v>
+        <v>130</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>104</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>16</v>
+        <v>131</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>195</v>
+        <v>107</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>105</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>106</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>107</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>19</v>
+        <v>134</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>108</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>109</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>21</v>
+        <v>136</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>110</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>22</v>
+        <v>137</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>111</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>23</v>
+        <v>138</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>112</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>113</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>114</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>26</v>
+        <v>141</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>27</v>
+        <v>142</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>116</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>194</v>
+        <v>106</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>11</v>
+        <v>144</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>29</v>
+        <v>145</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>118</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>30</v>
+        <v>146</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>119</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>190</v>
+        <v>102</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>120</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>196</v>
+        <v>108</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>121</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>33</v>
+        <v>149</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>191</v>
+        <v>103</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>122</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>197</v>
+        <v>109</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>123</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>35</v>
+        <v>152</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>125</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>36</v>
+        <v>153</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>126</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>37</v>
+        <v>154</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>127</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>38</v>
+        <v>155</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>128</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>39</v>
+        <v>156</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>129</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>40</v>
+        <v>157</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>131</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>41</v>
+        <v>158</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>132</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>42</v>
+        <v>159</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>133</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>43</v>
+        <v>160</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>134</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>44</v>
+        <v>161</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>135</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>45</v>
+        <v>162</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>136</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>46</v>
+        <v>163</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>196</v>
+        <v>108</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>47</v>
+        <v>164</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>138</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>48</v>
+        <v>165</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>139</v>
+        <v>51</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>140</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>50</v>
+        <v>167</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>197</v>
+        <v>109</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>141</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>51</v>
+        <v>168</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>142</v>
+        <v>54</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>52</v>
+        <v>169</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>143</v>
+        <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>53</v>
+        <v>170</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>196</v>
+        <v>108</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>144</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>54</v>
+        <v>171</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>145</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>55</v>
+        <v>172</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>146</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>56</v>
+        <v>173</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>147</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>57</v>
+        <v>174</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>141</v>
+        <v>53</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>58</v>
+        <v>175</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>148</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>59</v>
+        <v>176</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>203</v>
+        <v>115</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>149</v>
+        <v>61</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>60</v>
+        <v>177</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>150</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>61</v>
+        <v>178</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>198</v>
+        <v>110</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>151</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>62</v>
+        <v>179</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>152</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>153</v>
+        <v>65</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>63</v>
+        <v>181</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>154</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>42</v>
+        <v>182</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>155</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>12</v>
+        <v>183</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>156</v>
+        <v>68</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>64</v>
+        <v>184</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>157</v>
+        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>158</v>
+        <v>70</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>66</v>
+        <v>186</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>159</v>
+        <v>71</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>199</v>
+        <v>111</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>200</v>
+        <v>112</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>161</v>
+        <v>73</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>69</v>
+        <v>189</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>162</v>
+        <v>74</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>62</v>
+        <v>190</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>163</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>70</v>
+        <v>191</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>164</v>
+        <v>76</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>71</v>
+        <v>192</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>165</v>
+        <v>77</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>40</v>
+        <v>193</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>166</v>
+        <v>78</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>165</v>
+        <v>77</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>47</v>
+        <v>195</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>167</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>73</v>
+        <v>196</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>168</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>74</v>
+        <v>197</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>169</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>3</v>
+        <v>198</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>201</v>
+        <v>113</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>170</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>75</v>
+        <v>199</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>194</v>
+        <v>106</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>171</v>
+        <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>76</v>
+        <v>200</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>202</v>
+        <v>114</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>172</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>39</v>
+        <v>201</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>173</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>77</v>
+        <v>202</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>174</v>
+        <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>78</v>
+        <v>203</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>175</v>
+        <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>79</v>
+        <v>204</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>176</v>
+        <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>80</v>
+        <v>205</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>177</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>81</v>
+        <v>206</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>178</v>
+        <v>90</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>82</v>
+        <v>207</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>179</v>
+        <v>91</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>83</v>
+        <v>208</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>180</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>84</v>
+        <v>209</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>181</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>48</v>
+        <v>210</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>182</v>
+        <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>85</v>
+        <v>211</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>183</v>
+        <v>95</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>86</v>
+        <v>212</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>192</v>
+        <v>104</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>87</v>
+        <v>213</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>184</v>
+        <v>96</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>69</v>
+        <v>214</v>
       </c>
       <c r="B99" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>185</v>
+        <v>97</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>68</v>
+        <v>215</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>186</v>
+        <v>98</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
-        <v>88</v>
+        <v>216</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>187</v>
+        <v>99</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>89</v>
+        <v>217</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>188</v>
+        <v>100</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>90</v>
+        <v>218</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>